<commit_message>
Prepare CRM for Supabase and Vercel
</commit_message>
<xml_diff>
--- a/public/Plantilla_Prospectos_Sincro_CRM.xlsx
+++ b/public/Plantilla_Prospectos_Sincro_CRM.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga de prospectos" sheetId="1" r:id="Rbf2b989521d24ffa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rc8c90cd29c7b4009"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" r:id="R4a4104618f3e42a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga de prospectos" sheetId="1" r:id="R0f2f711d509a487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R8001957d96c34cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" r:id="Rae29cb3746df4477"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -43,13 +43,13 @@
     </x:font>
     <x:font>
       <x:sz val="9"/>
-      <x:color rgb="FF162438"/>
+      <x:color rgb="FF14202B"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="9"/>
-      <x:color rgb="FF162438"/>
+      <x:color rgb="FF14202B"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -66,13 +66,13 @@
     </x:font>
     <x:font>
       <x:sz val="10"/>
-      <x:color rgb="FF66758A"/>
+      <x:color rgb="FF6E7682"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF23330F"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -83,19 +83,13 @@
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
       <x:sz val="10"/>
-      <x:color rgb="FF162438"/>
+      <x:color rgb="FF14202B"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
-      <x:color rgb="FF162438"/>
+      <x:color rgb="FF14202B"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -108,17 +102,17 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF0A1726"/>
+        <x:fgColor rgb="FF0A2540"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEAF5FF"/>
+        <x:fgColor rgb="FFECECE7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF2C8FDE"/>
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -128,7 +122,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFB8E953"/>
+        <x:fgColor rgb="FFE9761D"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -136,41 +130,41 @@
     <x:border/>
     <x:border>
       <x:bottom style="thin">
-        <x:color rgb="FFE8EDF3"/>
+        <x:color rgb="FFEFEFEA"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:top style="thin">
-        <x:color rgb="FFE8EDF3"/>
+        <x:color rgb="FFEFEFEA"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFE8EDF3"/>
+        <x:color rgb="FFEFEFEA"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:top style="thin">
-        <x:color rgb="FFE8EDF3"/>
+        <x:color rgb="FFEFEFEA"/>
       </x:top>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFDDE5EE"/>
+        <x:color rgb="FFE4E3DD"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="FFDDE5EE"/>
+        <x:color rgb="FFE4E3DD"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFDDE5EE"/>
+        <x:color rgb="FFE4E3DD"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFDDE5EE"/>
+        <x:color rgb="FFE4E3DD"/>
       </x:bottom>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -182,31 +176,31 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -227,13 +221,13 @@
     <x:xf numFmtId="200" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -256,14 +250,15 @@
     <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -330,7 +325,7 @@
     <x:tableColumn id="8" name="Tanda"/>
     <x:tableColumn id="9" name="Notas"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -568,31 +563,31 @@
     </x:row>
     <x:row r="3" ht="8" customHeight="1"/>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="9" t="str">
+      <x:c r="A4" s="8" t="str">
         <x:v>Negocio</x:v>
       </x:c>
-      <x:c r="B4" s="9" t="str">
+      <x:c r="B4" s="8" t="str">
         <x:v>Email</x:v>
       </x:c>
-      <x:c r="C4" s="9" t="str">
+      <x:c r="C4" s="8" t="str">
         <x:v>Teléfono</x:v>
       </x:c>
-      <x:c r="D4" s="9" t="str">
+      <x:c r="D4" s="8" t="str">
         <x:v>Rubro</x:v>
       </x:c>
-      <x:c r="E4" s="9" t="str">
+      <x:c r="E4" s="8" t="str">
         <x:v>Responsable</x:v>
       </x:c>
-      <x:c r="F4" s="9" t="str">
+      <x:c r="F4" s="8" t="str">
         <x:v>Estado</x:v>
       </x:c>
-      <x:c r="G4" s="9" t="str">
+      <x:c r="G4" s="8" t="str">
         <x:v>Prioridad</x:v>
       </x:c>
-      <x:c r="H4" s="9" t="str">
+      <x:c r="H4" s="8" t="str">
         <x:v>Tanda</x:v>
       </x:c>
-      <x:c r="I4" s="9" t="str">
+      <x:c r="I4" s="8" t="str">
         <x:v>Notas</x:v>
       </x:c>
     </x:row>
@@ -1722,7 +1717,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fa74343624a43a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63460d9213d94ca6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1888,40 +1883,40 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="40" t="str">
+      <x:c r="A20" s="41" t="str">
         <x:v>Estudio Horizonte</x:v>
       </x:c>
-      <x:c r="B20" s="40" t="str">
+      <x:c r="B20" s="41" t="str">
         <x:v>hola@horizonte.com</x:v>
       </x:c>
-      <x:c r="C20" s="41" t="str">
+      <x:c r="C20" s="42" t="str">
         <x:v>5491144228899</x:v>
       </x:c>
-      <x:c r="D20" s="40" t="str">
+      <x:c r="D20" s="41" t="str">
         <x:v>Arquitectura</x:v>
       </x:c>
-      <x:c r="E20" s="40" t="str">
+      <x:c r="E20" s="41" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="F20" s="40" t="str">
+      <x:c r="F20" s="41" t="str">
         <x:v>Alta</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="40" t="str">
+      <x:c r="A21" s="41" t="str">
         <x:v>Mínimo válido</x:v>
       </x:c>
-      <x:c r="B21" s="40" t="str"/>
-      <x:c r="C21" s="41" t="str">
+      <x:c r="B21" s="41" t="str"/>
+      <x:c r="C21" s="42" t="str">
         <x:v>5491166778899</x:v>
       </x:c>
-      <x:c r="D21" s="40" t="str">
+      <x:c r="D21" s="41" t="str">
         <x:v>Gastronomía</x:v>
       </x:c>
-      <x:c r="E21" s="40" t="str">
+      <x:c r="E21" s="41" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="F21" s="40" t="str">
+      <x:c r="F21" s="41" t="str">
         <x:v>Media</x:v>
       </x:c>
     </x:row>
@@ -1950,90 +1945,90 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="47" t="str">
+      <x:c r="A1" s="48" t="str">
         <x:v>Responsables</x:v>
       </x:c>
-      <x:c r="B1" s="47" t="str">
+      <x:c r="B1" s="48" t="str">
         <x:v>Estados</x:v>
       </x:c>
-      <x:c r="C1" s="47" t="str">
+      <x:c r="C1" s="48" t="str">
         <x:v>Prioridades</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="46" t="str">
+      <x:c r="A2" s="47" t="str">
         <x:v>Franco</x:v>
       </x:c>
-      <x:c r="B2" s="46" t="str">
+      <x:c r="B2" s="47" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="C2" s="46" t="str">
+      <x:c r="C2" s="47" t="str">
         <x:v>Alta</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="46" t="str">
+      <x:c r="A3" s="47" t="str">
         <x:v>Equipo 2</x:v>
       </x:c>
-      <x:c r="B3" s="46" t="str">
+      <x:c r="B3" s="47" t="str">
         <x:v>Contactado</x:v>
       </x:c>
-      <x:c r="C3" s="46" t="str">
+      <x:c r="C3" s="47" t="str">
         <x:v>Media</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="46" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>Equipo 3</x:v>
       </x:c>
-      <x:c r="B4" s="46" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>Respondió</x:v>
       </x:c>
-      <x:c r="C4" s="46" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>Baja</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="46"/>
-      <x:c r="B5" s="46" t="str">
+      <x:c r="A5" s="47"/>
+      <x:c r="B5" s="47" t="str">
         <x:v>No respondió</x:v>
       </x:c>
-      <x:c r="C5" s="46"/>
+      <x:c r="C5" s="47"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="46"/>
-      <x:c r="B6" s="46" t="str">
+      <x:c r="A6" s="47"/>
+      <x:c r="B6" s="47" t="str">
         <x:v>No interesado</x:v>
       </x:c>
-      <x:c r="C6" s="46"/>
+      <x:c r="C6" s="47"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="46"/>
-      <x:c r="B7" s="46" t="str">
+      <x:c r="A7" s="47"/>
+      <x:c r="B7" s="47" t="str">
         <x:v>Propuesta enviada</x:v>
       </x:c>
-      <x:c r="C7" s="46"/>
+      <x:c r="C7" s="47"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="46"/>
-      <x:c r="B8" s="46" t="str">
+      <x:c r="A8" s="47"/>
+      <x:c r="B8" s="47" t="str">
         <x:v>Reunión agendada</x:v>
       </x:c>
-      <x:c r="C8" s="46"/>
+      <x:c r="C8" s="47"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="46"/>
-      <x:c r="B9" s="46" t="str">
+      <x:c r="A9" s="47"/>
+      <x:c r="B9" s="47" t="str">
         <x:v>Cerrado</x:v>
       </x:c>
-      <x:c r="C9" s="46"/>
+      <x:c r="C9" s="47"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="46"/>
-      <x:c r="B10" s="46" t="str">
+      <x:c r="A10" s="47"/>
+      <x:c r="B10" s="47" t="str">
         <x:v>Perdido</x:v>
       </x:c>
-      <x:c r="C10" s="46"/>
+      <x:c r="C10" s="47"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update Excel template owners
</commit_message>
<xml_diff>
--- a/public/Plantilla_Prospectos_Sincro_CRM.xlsx
+++ b/public/Plantilla_Prospectos_Sincro_CRM.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga de prospectos" sheetId="1" r:id="R0f2f711d509a487b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R8001957d96c34cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" r:id="Rae29cb3746df4477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga de prospectos" sheetId="1" r:id="R22681828be3841b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R83cfc92532db487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" r:id="R413bf0e7075f4155"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1717,7 +1717,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63460d9213d94ca6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cabc26d127249f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1968,7 +1968,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="47" t="str">
-        <x:v>Equipo 2</x:v>
+        <x:v>Teresa</x:v>
       </x:c>
       <x:c r="B3" s="47" t="str">
         <x:v>Contactado</x:v>
@@ -1979,7 +1979,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="47" t="str">
-        <x:v>Equipo 3</x:v>
+        <x:v>Laucha</x:v>
       </x:c>
       <x:c r="B4" s="47" t="str">
         <x:v>Respondió</x:v>

</xml_diff>

<commit_message>
Correct Excel owner name
</commit_message>
<xml_diff>
--- a/public/Plantilla_Prospectos_Sincro_CRM.xlsx
+++ b/public/Plantilla_Prospectos_Sincro_CRM.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga de prospectos" sheetId="1" r:id="R22681828be3841b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R83cfc92532db487e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" r:id="R413bf0e7075f4155"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga de prospectos" sheetId="1" r:id="Rd0ae2426171e47d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R5664493a3fb94c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" r:id="R16effedcdcf24d0d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1717,7 +1717,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cabc26d127249f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf46188cdbef54a4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1968,7 +1968,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="47" t="str">
-        <x:v>Teresa</x:v>
+        <x:v>Trezza</x:v>
       </x:c>
       <x:c r="B3" s="47" t="str">
         <x:v>Contactado</x:v>

</xml_diff>